<commit_message>
2025-01-25 JCI Insight Revisions
</commit_message>
<xml_diff>
--- a/tables/match-rate_specialty-degrees_stats.xlsx
+++ b/tables/match-rate_specialty-degrees_stats.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bcmedu-my.sharepoint.com/personal/u244834_bcm_edu/Documents/APSA/2024-07-29_Texas-STAR/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_93A8DCD88F79A8D366075C52F37BD2727AC6B517" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4522C0D4-B2EB-4722-B8E1-7CDAD01DA221}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="11_1CD9FFC98F79A8D366075C52F37BD2728AC0A657" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4421721C-7337-414A-867B-4F84D70B2FDC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="140">
   <si>
     <t>spec_degree</t>
   </si>
@@ -70,6 +83,9 @@
     <t>p.adj.signif</t>
   </si>
   <si>
+    <t>significant</t>
+  </si>
+  <si>
     <t>Anesthesiology_MD-MBA</t>
   </si>
   <si>
@@ -80,6 +96,9 @@
   </si>
   <si>
     <t>ns</t>
+  </si>
+  <si>
+    <t>not significant</t>
   </si>
   <si>
     <t>Anesthesiology_MD-MPH</t>
@@ -440,6 +459,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -457,12 +479,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -477,11 +505,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -786,21 +822,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P93"/>
+  <dimension ref="A1:Q93"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="15.42578125" customWidth="1"/>
+    <col min="9" max="9" width="17" style="3" customWidth="1"/>
+    <col min="13" max="13" width="11.140625" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
+    <col min="15" max="15" width="10.140625" customWidth="1"/>
+    <col min="16" max="16" width="13.5703125" customWidth="1"/>
+    <col min="17" max="17" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -816,7 +857,7 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -825,7 +866,7 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
@@ -849,16 +890,19 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2">
         <v>35</v>
@@ -866,7 +910,7 @@
       <c r="E2">
         <v>6</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="5">
         <v>85.365853658536579</v>
       </c>
       <c r="G2">
@@ -875,7 +919,7 @@
       <c r="H2">
         <v>167</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="3">
         <v>91.270256142185048</v>
       </c>
       <c r="J2">
@@ -897,18 +941,21 @@
         <v>0.622</v>
       </c>
       <c r="P2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D3">
         <v>68</v>
@@ -916,7 +963,7 @@
       <c r="E3">
         <v>8</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="5">
         <v>89.473684210526315</v>
       </c>
       <c r="G3">
@@ -925,7 +972,7 @@
       <c r="H3">
         <v>167</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="3">
         <v>91.270256142185048</v>
       </c>
       <c r="J3">
@@ -947,18 +994,21 @@
         <v>0.622</v>
       </c>
       <c r="P3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D4">
         <v>143</v>
@@ -966,7 +1016,7 @@
       <c r="E4">
         <v>16</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="5">
         <v>89.937106918238996</v>
       </c>
       <c r="G4">
@@ -975,7 +1025,7 @@
       <c r="H4">
         <v>167</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="3">
         <v>91.270256142185048</v>
       </c>
       <c r="J4">
@@ -997,18 +1047,21 @@
         <v>0.622</v>
       </c>
       <c r="P4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D5">
         <v>47</v>
@@ -1016,7 +1069,7 @@
       <c r="E5">
         <v>2</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="5">
         <v>95.918367346938766</v>
       </c>
       <c r="G5">
@@ -1025,7 +1078,7 @@
       <c r="H5">
         <v>167</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="3">
         <v>91.270256142185048</v>
       </c>
       <c r="J5">
@@ -1047,18 +1100,21 @@
         <v>0.622</v>
       </c>
       <c r="P5" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
       </c>
       <c r="D6">
         <v>3</v>
@@ -1066,7 +1122,7 @@
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="5">
         <v>100</v>
       </c>
       <c r="G6">
@@ -1075,14 +1131,14 @@
       <c r="H6">
         <v>9</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="3">
         <v>95.544554455445535</v>
       </c>
       <c r="J6">
         <v>205</v>
       </c>
       <c r="K6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L6">
         <v>1</v>
@@ -1091,24 +1147,27 @@
         <v>1.7539861272656519E-2</v>
       </c>
       <c r="N6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O6">
         <v>1</v>
       </c>
       <c r="P6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
         <v>29</v>
       </c>
-      <c r="B7" t="s">
-        <v>27</v>
-      </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -1116,7 +1175,7 @@
       <c r="E7">
         <v>1</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="5">
         <v>80</v>
       </c>
       <c r="G7">
@@ -1125,7 +1184,7 @@
       <c r="H7">
         <v>9</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="3">
         <v>95.544554455445535</v>
       </c>
       <c r="J7">
@@ -1147,18 +1206,21 @@
         <v>0.98</v>
       </c>
       <c r="P7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D8">
         <v>12</v>
@@ -1166,7 +1228,7 @@
       <c r="E8">
         <v>0</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="5">
         <v>100</v>
       </c>
       <c r="G8">
@@ -1175,14 +1237,14 @@
       <c r="H8">
         <v>9</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="3">
         <v>95.544554455445535</v>
       </c>
       <c r="J8">
         <v>214</v>
       </c>
       <c r="K8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L8">
         <v>1</v>
@@ -1191,24 +1253,27 @@
         <v>0.1078336279188465</v>
       </c>
       <c r="N8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O8">
         <v>1</v>
       </c>
       <c r="P8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" t="s">
         <v>27</v>
-      </c>
-      <c r="C9" t="s">
-        <v>25</v>
       </c>
       <c r="D9">
         <v>29</v>
@@ -1216,7 +1281,7 @@
       <c r="E9">
         <v>0</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="5">
         <v>100</v>
       </c>
       <c r="G9">
@@ -1225,14 +1290,14 @@
       <c r="H9">
         <v>9</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="3">
         <v>95.544554455445535</v>
       </c>
       <c r="J9">
         <v>231</v>
       </c>
       <c r="K9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L9">
         <v>0.60699999999999998</v>
@@ -1241,24 +1306,27 @@
         <v>0.27956456342969649</v>
       </c>
       <c r="N9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O9">
         <v>1</v>
       </c>
       <c r="P9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" t="s">
-        <v>18</v>
       </c>
       <c r="D10">
         <v>16</v>
@@ -1266,7 +1334,7 @@
       <c r="E10">
         <v>3</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="5">
         <v>84.210526315789465</v>
       </c>
       <c r="G10">
@@ -1275,7 +1343,7 @@
       <c r="H10">
         <v>95</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="3">
         <v>83.732876712328761</v>
       </c>
       <c r="J10">
@@ -1297,18 +1365,21 @@
         <v>1</v>
       </c>
       <c r="P10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D11">
         <v>17</v>
@@ -1316,7 +1387,7 @@
       <c r="E11">
         <v>3</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="5">
         <v>85</v>
       </c>
       <c r="G11">
@@ -1325,7 +1396,7 @@
       <c r="H11">
         <v>95</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="3">
         <v>83.732876712328761</v>
       </c>
       <c r="J11">
@@ -1347,18 +1418,21 @@
         <v>1</v>
       </c>
       <c r="P11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" t="s">
         <v>35</v>
       </c>
-      <c r="B12" t="s">
-        <v>33</v>
-      </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D12">
         <v>37</v>
@@ -1366,7 +1440,7 @@
       <c r="E12">
         <v>9</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="5">
         <v>80.434782608695656</v>
       </c>
       <c r="G12">
@@ -1375,7 +1449,7 @@
       <c r="H12">
         <v>95</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="3">
         <v>83.732876712328761</v>
       </c>
       <c r="J12">
@@ -1397,18 +1471,21 @@
         <v>1</v>
       </c>
       <c r="P12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D13">
         <v>35</v>
@@ -1416,7 +1493,7 @@
       <c r="E13">
         <v>6</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="5">
         <v>85.365853658536579</v>
       </c>
       <c r="G13">
@@ -1425,7 +1502,7 @@
       <c r="H13">
         <v>95</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="3">
         <v>83.732876712328761</v>
       </c>
       <c r="J13">
@@ -1447,18 +1524,21 @@
         <v>1</v>
       </c>
       <c r="P13" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" t="s">
-        <v>18</v>
       </c>
       <c r="D14">
         <v>43</v>
@@ -1466,7 +1546,7 @@
       <c r="E14">
         <v>6</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="5">
         <v>87.755102040816325</v>
       </c>
       <c r="G14">
@@ -1475,7 +1555,7 @@
       <c r="H14">
         <v>226</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="3">
         <v>91.307692307692307</v>
       </c>
       <c r="J14">
@@ -1497,18 +1577,21 @@
         <v>0.73</v>
       </c>
       <c r="P14" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D15">
         <v>139</v>
@@ -1516,7 +1599,7 @@
       <c r="E15">
         <v>9</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="5">
         <v>93.918918918918919</v>
       </c>
       <c r="G15">
@@ -1525,7 +1608,7 @@
       <c r="H15">
         <v>226</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="3">
         <v>91.307692307692307</v>
       </c>
       <c r="J15">
@@ -1547,18 +1630,21 @@
         <v>0.72599999999999998</v>
       </c>
       <c r="P15" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" t="s">
         <v>40</v>
       </c>
-      <c r="B16" t="s">
-        <v>38</v>
-      </c>
       <c r="C16" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D16">
         <v>200</v>
@@ -1566,7 +1652,7 @@
       <c r="E16">
         <v>26</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="5">
         <v>88.495575221238937</v>
       </c>
       <c r="G16">
@@ -1575,7 +1661,7 @@
       <c r="H16">
         <v>226</v>
       </c>
-      <c r="I16">
+      <c r="I16" s="3">
         <v>91.307692307692307</v>
       </c>
       <c r="J16">
@@ -1597,18 +1683,21 @@
         <v>0.69299999999999995</v>
       </c>
       <c r="P16" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D17">
         <v>31</v>
@@ -1616,7 +1705,7 @@
       <c r="E17">
         <v>4</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="5">
         <v>88.571428571428569</v>
       </c>
       <c r="G17">
@@ -1625,7 +1714,7 @@
       <c r="H17">
         <v>226</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="3">
         <v>91.307692307692307</v>
       </c>
       <c r="J17">
@@ -1647,18 +1736,21 @@
         <v>0.77300000000000002</v>
       </c>
       <c r="P17" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" t="s">
-        <v>18</v>
       </c>
       <c r="D18">
         <v>25</v>
@@ -1666,7 +1758,7 @@
       <c r="E18">
         <v>7</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="5">
         <v>78.125</v>
       </c>
       <c r="G18">
@@ -1675,7 +1767,7 @@
       <c r="H18">
         <v>235</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="3">
         <v>90.474260235103372</v>
       </c>
       <c r="J18">
@@ -1697,18 +1789,21 @@
         <v>0.28799999999999998</v>
       </c>
       <c r="P18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D19">
         <v>202</v>
@@ -1716,7 +1811,7 @@
       <c r="E19">
         <v>20</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="5">
         <v>90.990990990990994</v>
       </c>
       <c r="G19">
@@ -1725,7 +1820,7 @@
       <c r="H19">
         <v>235</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="3">
         <v>90.474260235103372</v>
       </c>
       <c r="J19">
@@ -1747,18 +1842,21 @@
         <v>1</v>
       </c>
       <c r="P19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" t="s">
         <v>45</v>
       </c>
-      <c r="B20" t="s">
-        <v>43</v>
-      </c>
       <c r="C20" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D20">
         <v>134</v>
@@ -1766,7 +1864,7 @@
       <c r="E20">
         <v>18</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="5">
         <v>88.157894736842096</v>
       </c>
       <c r="G20">
@@ -1775,7 +1873,7 @@
       <c r="H20">
         <v>235</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="3">
         <v>90.474260235103372</v>
       </c>
       <c r="J20">
@@ -1797,18 +1895,21 @@
         <v>0.75700000000000001</v>
       </c>
       <c r="P20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B21" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C21" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D21">
         <v>18</v>
@@ -1816,7 +1917,7 @@
       <c r="E21">
         <v>2</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="5">
         <v>90</v>
       </c>
       <c r="G21">
@@ -1825,7 +1926,7 @@
       <c r="H21">
         <v>235</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="3">
         <v>90.474260235103372</v>
       </c>
       <c r="J21">
@@ -1847,18 +1948,21 @@
         <v>1</v>
       </c>
       <c r="P21" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" t="s">
-        <v>48</v>
-      </c>
-      <c r="C22" t="s">
-        <v>18</v>
       </c>
       <c r="D22">
         <v>7</v>
@@ -1866,7 +1970,7 @@
       <c r="E22">
         <v>1</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="5">
         <v>87.5</v>
       </c>
       <c r="G22">
@@ -1875,7 +1979,7 @@
       <c r="H22">
         <v>66</v>
       </c>
-      <c r="I22">
+      <c r="I22" s="3">
         <v>89.81481481481481</v>
       </c>
       <c r="J22">
@@ -1897,18 +2001,21 @@
         <v>0.91700000000000004</v>
       </c>
       <c r="P22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D23">
         <v>52</v>
@@ -1916,7 +2023,7 @@
       <c r="E23">
         <v>4</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="5">
         <v>92.857142857142861</v>
       </c>
       <c r="G23">
@@ -1925,7 +2032,7 @@
       <c r="H23">
         <v>66</v>
       </c>
-      <c r="I23">
+      <c r="I23" s="3">
         <v>89.81481481481481</v>
       </c>
       <c r="J23">
@@ -1947,18 +2054,21 @@
         <v>0.91700000000000004</v>
       </c>
       <c r="P23" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" t="s">
         <v>50</v>
       </c>
-      <c r="B24" t="s">
-        <v>48</v>
-      </c>
       <c r="C24" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D24">
         <v>46</v>
@@ -1966,7 +2076,7 @@
       <c r="E24">
         <v>4</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="5">
         <v>92</v>
       </c>
       <c r="G24">
@@ -1975,7 +2085,7 @@
       <c r="H24">
         <v>66</v>
       </c>
-      <c r="I24">
+      <c r="I24" s="3">
         <v>89.81481481481481</v>
       </c>
       <c r="J24">
@@ -1997,18 +2107,21 @@
         <v>1</v>
       </c>
       <c r="P24" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C25" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D25">
         <v>10</v>
@@ -2016,7 +2129,7 @@
       <c r="E25">
         <v>2</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="5">
         <v>83.333333333333343</v>
       </c>
       <c r="G25">
@@ -2025,7 +2138,7 @@
       <c r="H25">
         <v>66</v>
       </c>
-      <c r="I25">
+      <c r="I25" s="3">
         <v>89.81481481481481</v>
       </c>
       <c r="J25">
@@ -2047,18 +2160,21 @@
         <v>0.91700000000000004</v>
       </c>
       <c r="P25" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>52</v>
-      </c>
-      <c r="B26" t="s">
-        <v>53</v>
-      </c>
-      <c r="C26" t="s">
-        <v>18</v>
       </c>
       <c r="D26">
         <v>94</v>
@@ -2066,7 +2182,7 @@
       <c r="E26">
         <v>10</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="5">
         <v>90.384615384615387</v>
       </c>
       <c r="G26">
@@ -2075,7 +2191,7 @@
       <c r="H26">
         <v>352</v>
       </c>
-      <c r="I26">
+      <c r="I26" s="3">
         <v>92.791316813434364</v>
       </c>
       <c r="J26">
@@ -2097,18 +2213,21 @@
         <v>0.79200000000000004</v>
       </c>
       <c r="P26" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B27" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D27">
         <v>260</v>
@@ -2116,7 +2235,7 @@
       <c r="E27">
         <v>30</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="5">
         <v>89.65517241379311</v>
       </c>
       <c r="G27">
@@ -2125,7 +2244,7 @@
       <c r="H27">
         <v>352</v>
       </c>
-      <c r="I27">
+      <c r="I27" s="3">
         <v>92.791316813434364</v>
       </c>
       <c r="J27">
@@ -2147,18 +2266,21 @@
         <v>0.316</v>
       </c>
       <c r="P27" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" t="s">
         <v>55</v>
       </c>
-      <c r="B28" t="s">
-        <v>53</v>
-      </c>
       <c r="C28" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D28">
         <v>348</v>
@@ -2166,7 +2288,7 @@
       <c r="E28">
         <v>46</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="5">
         <v>88.324873096446694</v>
       </c>
       <c r="G28">
@@ -2175,7 +2297,7 @@
       <c r="H28">
         <v>352</v>
       </c>
-      <c r="I28">
+      <c r="I28" s="3">
         <v>92.791316813434364</v>
       </c>
       <c r="J28">
@@ -2197,18 +2319,21 @@
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="P28" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B29" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C29" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D29">
         <v>254</v>
@@ -2216,7 +2341,7 @@
       <c r="E29">
         <v>23</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="5">
         <v>91.696750902527086</v>
       </c>
       <c r="G29">
@@ -2225,7 +2350,7 @@
       <c r="H29">
         <v>352</v>
       </c>
-      <c r="I29">
+      <c r="I29" s="3">
         <v>92.791316813434364</v>
       </c>
       <c r="J29">
@@ -2247,18 +2372,21 @@
         <v>0.79200000000000004</v>
       </c>
       <c r="P29" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" t="s">
+        <v>61</v>
+      </c>
+      <c r="C30" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>58</v>
-      </c>
-      <c r="B30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C30" t="s">
-        <v>18</v>
       </c>
       <c r="D30">
         <v>2</v>
@@ -2266,7 +2394,7 @@
       <c r="E30">
         <v>0</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="5">
         <v>100</v>
       </c>
       <c r="G30">
@@ -2275,14 +2403,14 @@
       <c r="H30">
         <v>34</v>
       </c>
-      <c r="I30">
+      <c r="I30" s="3">
         <v>86.345381526104418</v>
       </c>
       <c r="J30">
         <v>251</v>
       </c>
       <c r="K30" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L30">
         <v>1</v>
@@ -2291,24 +2419,27 @@
         <v>2.9137629261578629E-2</v>
       </c>
       <c r="N30" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O30">
         <v>1</v>
       </c>
       <c r="P30" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B31" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C31" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D31">
         <v>8</v>
@@ -2316,7 +2447,7 @@
       <c r="E31">
         <v>0</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="5">
         <v>100</v>
       </c>
       <c r="G31">
@@ -2325,14 +2456,14 @@
       <c r="H31">
         <v>34</v>
       </c>
-      <c r="I31">
+      <c r="I31" s="3">
         <v>86.345381526104418</v>
       </c>
       <c r="J31">
         <v>257</v>
       </c>
       <c r="K31" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L31">
         <v>0.60199999999999998</v>
@@ -2341,24 +2472,27 @@
         <v>0.25700164923035701</v>
       </c>
       <c r="N31" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O31">
         <v>1</v>
       </c>
       <c r="P31" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" t="s">
         <v>61</v>
       </c>
-      <c r="B32" t="s">
-        <v>59</v>
-      </c>
       <c r="C32" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D32">
         <v>38</v>
@@ -2366,7 +2500,7 @@
       <c r="E32">
         <v>7</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="5">
         <v>84.444444444444443</v>
       </c>
       <c r="G32">
@@ -2375,7 +2509,7 @@
       <c r="H32">
         <v>34</v>
       </c>
-      <c r="I32">
+      <c r="I32" s="3">
         <v>86.345381526104418</v>
       </c>
       <c r="J32">
@@ -2397,18 +2531,21 @@
         <v>1</v>
       </c>
       <c r="P32" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B33" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C33" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D33">
         <v>29</v>
@@ -2416,7 +2553,7 @@
       <c r="E33">
         <v>3</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="5">
         <v>90.625</v>
       </c>
       <c r="G33">
@@ -2425,7 +2562,7 @@
       <c r="H33">
         <v>34</v>
       </c>
-      <c r="I33">
+      <c r="I33" s="3">
         <v>86.345381526104418</v>
       </c>
       <c r="J33">
@@ -2447,18 +2584,21 @@
         <v>1</v>
       </c>
       <c r="P33" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B34" t="s">
-        <v>64</v>
-      </c>
-      <c r="C34" t="s">
-        <v>18</v>
       </c>
       <c r="D34">
         <v>10</v>
@@ -2466,7 +2606,7 @@
       <c r="E34">
         <v>1</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="5">
         <v>90.909090909090907</v>
       </c>
       <c r="G34">
@@ -2475,7 +2615,7 @@
       <c r="H34">
         <v>39</v>
       </c>
-      <c r="I34">
+      <c r="I34" s="3">
         <v>94.388489208633104</v>
       </c>
       <c r="J34">
@@ -2497,18 +2637,21 @@
         <v>1</v>
       </c>
       <c r="P34" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B35" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C35" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D35">
         <v>39</v>
@@ -2516,7 +2659,7 @@
       <c r="E35">
         <v>2</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="5">
         <v>95.121951219512198</v>
       </c>
       <c r="G35">
@@ -2525,7 +2668,7 @@
       <c r="H35">
         <v>39</v>
       </c>
-      <c r="I35">
+      <c r="I35" s="3">
         <v>94.388489208633104</v>
       </c>
       <c r="J35">
@@ -2547,18 +2690,21 @@
         <v>1</v>
       </c>
       <c r="P35" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" t="s">
         <v>66</v>
       </c>
-      <c r="B36" t="s">
-        <v>64</v>
-      </c>
       <c r="C36" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D36">
         <v>67</v>
@@ -2566,7 +2712,7 @@
       <c r="E36">
         <v>4</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="5">
         <v>94.366197183098592</v>
       </c>
       <c r="G36">
@@ -2575,7 +2721,7 @@
       <c r="H36">
         <v>39</v>
       </c>
-      <c r="I36">
+      <c r="I36" s="3">
         <v>94.388489208633104</v>
       </c>
       <c r="J36">
@@ -2597,18 +2743,21 @@
         <v>1</v>
       </c>
       <c r="P36" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B37" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C37" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D37">
         <v>81</v>
@@ -2616,7 +2765,7 @@
       <c r="E37">
         <v>3</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="5">
         <v>96.428571428571431</v>
       </c>
       <c r="G37">
@@ -2625,7 +2774,7 @@
       <c r="H37">
         <v>39</v>
       </c>
-      <c r="I37">
+      <c r="I37" s="3">
         <v>94.388489208633104</v>
       </c>
       <c r="J37">
@@ -2647,18 +2796,21 @@
         <v>1</v>
       </c>
       <c r="P37" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>70</v>
+      </c>
+      <c r="B38" t="s">
+        <v>71</v>
+      </c>
+      <c r="C38" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>68</v>
-      </c>
-      <c r="B38" t="s">
-        <v>69</v>
-      </c>
-      <c r="C38" t="s">
-        <v>18</v>
       </c>
       <c r="D38">
         <v>22</v>
@@ -2666,7 +2818,7 @@
       <c r="E38">
         <v>0</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="5">
         <v>100</v>
       </c>
       <c r="G38">
@@ -2675,14 +2827,14 @@
       <c r="H38">
         <v>265</v>
       </c>
-      <c r="I38">
+      <c r="I38" s="3">
         <v>87.160852713178301</v>
       </c>
       <c r="J38">
         <v>2086</v>
       </c>
       <c r="K38" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L38">
         <v>0.1</v>
@@ -2691,24 +2843,27 @@
         <v>0.80080457193057364</v>
       </c>
       <c r="N38" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O38">
         <v>0.2</v>
       </c>
       <c r="P38" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B39" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C39" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D39">
         <v>194</v>
@@ -2716,7 +2871,7 @@
       <c r="E39">
         <v>15</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="5">
         <v>92.822966507177028</v>
       </c>
       <c r="G39">
@@ -2725,7 +2880,7 @@
       <c r="H39">
         <v>265</v>
       </c>
-      <c r="I39">
+      <c r="I39" s="3">
         <v>87.160852713178301</v>
       </c>
       <c r="J39">
@@ -2747,18 +2902,21 @@
         <v>0.15</v>
       </c>
       <c r="P39" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>73</v>
+      </c>
+      <c r="B40" t="s">
         <v>71</v>
       </c>
-      <c r="B40" t="s">
-        <v>69</v>
-      </c>
       <c r="C40" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D40">
         <v>144</v>
@@ -2766,7 +2924,7 @@
       <c r="E40">
         <v>21</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="5">
         <v>87.272727272727266</v>
       </c>
       <c r="G40">
@@ -2775,7 +2933,7 @@
       <c r="H40">
         <v>265</v>
       </c>
-      <c r="I40">
+      <c r="I40" s="3">
         <v>87.160852713178301</v>
       </c>
       <c r="J40">
@@ -2797,18 +2955,21 @@
         <v>1</v>
       </c>
       <c r="P40" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B41" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C41" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D41">
         <v>28</v>
@@ -2816,7 +2977,7 @@
       <c r="E41">
         <v>6</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="5">
         <v>82.35294117647058</v>
       </c>
       <c r="G41">
@@ -2825,7 +2986,7 @@
       <c r="H41">
         <v>265</v>
       </c>
-      <c r="I41">
+      <c r="I41" s="3">
         <v>87.160852713178301</v>
       </c>
       <c r="J41">
@@ -2847,18 +3008,21 @@
         <v>0.48299999999999998</v>
       </c>
       <c r="P41" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>75</v>
+      </c>
+      <c r="B42" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>73</v>
-      </c>
-      <c r="B42" t="s">
-        <v>74</v>
-      </c>
-      <c r="C42" t="s">
-        <v>18</v>
       </c>
       <c r="D42">
         <v>14</v>
@@ -2866,7 +3030,7 @@
       <c r="E42">
         <v>3</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="5">
         <v>82.35294117647058</v>
       </c>
       <c r="G42">
@@ -2875,7 +3039,7 @@
       <c r="H42">
         <v>77</v>
       </c>
-      <c r="I42">
+      <c r="I42" s="3">
         <v>88.208269525267994</v>
       </c>
       <c r="J42">
@@ -2897,18 +3061,21 @@
         <v>1</v>
       </c>
       <c r="P42" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B43" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C43" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D43">
         <v>21</v>
@@ -2916,7 +3083,7 @@
       <c r="E43">
         <v>3</v>
       </c>
-      <c r="F43">
+      <c r="F43" s="5">
         <v>87.5</v>
       </c>
       <c r="G43">
@@ -2925,7 +3092,7 @@
       <c r="H43">
         <v>77</v>
       </c>
-      <c r="I43">
+      <c r="I43" s="3">
         <v>88.208269525267994</v>
       </c>
       <c r="J43">
@@ -2947,18 +3114,21 @@
         <v>1</v>
       </c>
       <c r="P43" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>78</v>
+      </c>
+      <c r="B44" t="s">
         <v>76</v>
       </c>
-      <c r="B44" t="s">
-        <v>74</v>
-      </c>
       <c r="C44" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D44">
         <v>51</v>
@@ -2966,7 +3136,7 @@
       <c r="E44">
         <v>5</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="5">
         <v>91.071428571428569</v>
       </c>
       <c r="G44">
@@ -2975,7 +3145,7 @@
       <c r="H44">
         <v>77</v>
       </c>
-      <c r="I44">
+      <c r="I44" s="3">
         <v>88.208269525267994</v>
       </c>
       <c r="J44">
@@ -2997,18 +3167,21 @@
         <v>1</v>
       </c>
       <c r="P44" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B45" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C45" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D45">
         <v>20</v>
@@ -3016,7 +3189,7 @@
       <c r="E45">
         <v>2</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="5">
         <v>90.909090909090907</v>
       </c>
       <c r="G45">
@@ -3025,7 +3198,7 @@
       <c r="H45">
         <v>77</v>
       </c>
-      <c r="I45">
+      <c r="I45" s="3">
         <v>88.208269525267994</v>
       </c>
       <c r="J45">
@@ -3047,18 +3220,21 @@
         <v>1</v>
       </c>
       <c r="P45" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>80</v>
+      </c>
+      <c r="B46" t="s">
+        <v>81</v>
+      </c>
+      <c r="C46" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>78</v>
-      </c>
-      <c r="B46" t="s">
-        <v>79</v>
-      </c>
-      <c r="C46" t="s">
-        <v>18</v>
       </c>
       <c r="D46">
         <v>21</v>
@@ -3066,7 +3242,7 @@
       <c r="E46">
         <v>2</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="5">
         <v>91.304347826086953</v>
       </c>
       <c r="G46">
@@ -3075,7 +3251,7 @@
       <c r="H46">
         <v>185</v>
       </c>
-      <c r="I46">
+      <c r="I46" s="3">
         <v>84.660033167495854</v>
       </c>
       <c r="J46">
@@ -3097,18 +3273,21 @@
         <v>0.93600000000000005</v>
       </c>
       <c r="P46" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B47" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C47" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D47">
         <v>27</v>
@@ -3116,7 +3295,7 @@
       <c r="E47">
         <v>6</v>
       </c>
-      <c r="F47">
+      <c r="F47" s="5">
         <v>81.818181818181827</v>
       </c>
       <c r="G47">
@@ -3125,7 +3304,7 @@
       <c r="H47">
         <v>185</v>
       </c>
-      <c r="I47">
+      <c r="I47" s="3">
         <v>84.660033167495854</v>
       </c>
       <c r="J47">
@@ -3147,18 +3326,21 @@
         <v>0.93600000000000005</v>
       </c>
       <c r="P47" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>83</v>
+      </c>
+      <c r="B48" t="s">
         <v>81</v>
       </c>
-      <c r="B48" t="s">
-        <v>79</v>
-      </c>
       <c r="C48" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D48">
         <v>94</v>
@@ -3166,7 +3348,7 @@
       <c r="E48">
         <v>25</v>
       </c>
-      <c r="F48">
+      <c r="F48" s="5">
         <v>78.991596638655466</v>
       </c>
       <c r="G48">
@@ -3175,7 +3357,7 @@
       <c r="H48">
         <v>185</v>
       </c>
-      <c r="I48">
+      <c r="I48" s="3">
         <v>84.660033167495854</v>
       </c>
       <c r="J48">
@@ -3197,18 +3379,21 @@
         <v>0.93600000000000005</v>
       </c>
       <c r="P48" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B49" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C49" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D49">
         <v>11</v>
@@ -3216,7 +3401,7 @@
       <c r="E49">
         <v>1</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="5">
         <v>91.666666666666657</v>
       </c>
       <c r="G49">
@@ -3225,7 +3410,7 @@
       <c r="H49">
         <v>185</v>
       </c>
-      <c r="I49">
+      <c r="I49" s="3">
         <v>84.660033167495854</v>
       </c>
       <c r="J49">
@@ -3247,18 +3432,21 @@
         <v>1</v>
       </c>
       <c r="P49" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>85</v>
+      </c>
+      <c r="B50" t="s">
+        <v>86</v>
+      </c>
+      <c r="C50" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>83</v>
-      </c>
-      <c r="B50" t="s">
-        <v>84</v>
-      </c>
-      <c r="C50" t="s">
-        <v>18</v>
       </c>
       <c r="D50">
         <v>7</v>
@@ -3266,7 +3454,7 @@
       <c r="E50">
         <v>6</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="5">
         <v>53.846153846153847</v>
       </c>
       <c r="G50">
@@ -3275,7 +3463,7 @@
       <c r="H50">
         <v>99</v>
       </c>
-      <c r="I50">
+      <c r="I50" s="3">
         <v>83.134582623509374</v>
       </c>
       <c r="J50">
@@ -3297,18 +3485,21 @@
         <v>0.15</v>
       </c>
       <c r="P50" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B51" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C51" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D51">
         <v>20</v>
@@ -3316,7 +3507,7 @@
       <c r="E51">
         <v>5</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="5">
         <v>80</v>
       </c>
       <c r="G51">
@@ -3325,7 +3516,7 @@
       <c r="H51">
         <v>99</v>
       </c>
-      <c r="I51">
+      <c r="I51" s="3">
         <v>83.134582623509374</v>
       </c>
       <c r="J51">
@@ -3347,18 +3538,21 @@
         <v>0.66200000000000003</v>
       </c>
       <c r="P51" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>88</v>
+      </c>
+      <c r="B52" t="s">
         <v>86</v>
       </c>
-      <c r="B52" t="s">
-        <v>84</v>
-      </c>
       <c r="C52" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D52">
         <v>40</v>
@@ -3366,7 +3560,7 @@
       <c r="E52">
         <v>11</v>
       </c>
-      <c r="F52">
+      <c r="F52" s="5">
         <v>78.431372549019613</v>
       </c>
       <c r="G52">
@@ -3375,7 +3569,7 @@
       <c r="H52">
         <v>99</v>
       </c>
-      <c r="I52">
+      <c r="I52" s="3">
         <v>83.134582623509374</v>
       </c>
       <c r="J52">
@@ -3397,18 +3591,21 @@
         <v>0.60499999999999998</v>
       </c>
       <c r="P52" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q52" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B53" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C53" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D53">
         <v>13</v>
@@ -3416,7 +3613,7 @@
       <c r="E53">
         <v>1</v>
       </c>
-      <c r="F53">
+      <c r="F53" s="5">
         <v>92.857142857142861</v>
       </c>
       <c r="G53">
@@ -3425,7 +3622,7 @@
       <c r="H53">
         <v>99</v>
       </c>
-      <c r="I53">
+      <c r="I53" s="3">
         <v>83.134582623509374</v>
       </c>
       <c r="J53">
@@ -3447,18 +3644,21 @@
         <v>0.60499999999999998</v>
       </c>
       <c r="P53" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q53" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>90</v>
+      </c>
+      <c r="B54" t="s">
+        <v>91</v>
+      </c>
+      <c r="C54" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>88</v>
-      </c>
-      <c r="B54" t="s">
-        <v>89</v>
-      </c>
-      <c r="C54" t="s">
-        <v>18</v>
       </c>
       <c r="D54">
         <v>2</v>
@@ -3466,7 +3666,7 @@
       <c r="E54">
         <v>0</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="5">
         <v>100</v>
       </c>
       <c r="G54">
@@ -3475,14 +3675,14 @@
       <c r="H54">
         <v>22</v>
       </c>
-      <c r="I54">
+      <c r="I54" s="3">
         <v>91.603053435114504</v>
       </c>
       <c r="J54">
         <v>264</v>
       </c>
       <c r="K54" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L54">
         <v>1</v>
@@ -3491,24 +3691,27 @@
         <v>1.6766159872556339E-2</v>
       </c>
       <c r="N54" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O54">
         <v>1</v>
       </c>
       <c r="P54" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B55" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C55" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D55">
         <v>16</v>
@@ -3516,7 +3719,7 @@
       <c r="E55">
         <v>2</v>
       </c>
-      <c r="F55">
+      <c r="F55" s="5">
         <v>88.888888888888886</v>
       </c>
       <c r="G55">
@@ -3525,7 +3728,7 @@
       <c r="H55">
         <v>22</v>
       </c>
-      <c r="I55">
+      <c r="I55" s="3">
         <v>91.603053435114504</v>
       </c>
       <c r="J55">
@@ -3547,18 +3750,21 @@
         <v>1</v>
       </c>
       <c r="P55" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>93</v>
+      </c>
+      <c r="B56" t="s">
         <v>91</v>
       </c>
-      <c r="B56" t="s">
-        <v>89</v>
-      </c>
       <c r="C56" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D56">
         <v>40</v>
@@ -3566,7 +3772,7 @@
       <c r="E56">
         <v>4</v>
       </c>
-      <c r="F56">
+      <c r="F56" s="5">
         <v>90.909090909090907</v>
       </c>
       <c r="G56">
@@ -3575,7 +3781,7 @@
       <c r="H56">
         <v>22</v>
       </c>
-      <c r="I56">
+      <c r="I56" s="3">
         <v>91.603053435114504</v>
       </c>
       <c r="J56">
@@ -3597,18 +3803,21 @@
         <v>1</v>
       </c>
       <c r="P56" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B57" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C57" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D57">
         <v>69</v>
@@ -3616,7 +3825,7 @@
       <c r="E57">
         <v>7</v>
       </c>
-      <c r="F57">
+      <c r="F57" s="5">
         <v>90.789473684210535</v>
       </c>
       <c r="G57">
@@ -3625,7 +3834,7 @@
       <c r="H57">
         <v>22</v>
       </c>
-      <c r="I57">
+      <c r="I57" s="3">
         <v>91.603053435114504</v>
       </c>
       <c r="J57">
@@ -3647,18 +3856,21 @@
         <v>1</v>
       </c>
       <c r="P57" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>95</v>
+      </c>
+      <c r="B58" t="s">
+        <v>96</v>
+      </c>
+      <c r="C58" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>93</v>
-      </c>
-      <c r="B58" t="s">
-        <v>94</v>
-      </c>
-      <c r="C58" t="s">
-        <v>18</v>
       </c>
       <c r="D58">
         <v>27</v>
@@ -3666,7 +3878,7 @@
       <c r="E58">
         <v>4</v>
       </c>
-      <c r="F58">
+      <c r="F58" s="5">
         <v>87.096774193548384</v>
       </c>
       <c r="G58">
@@ -3675,7 +3887,7 @@
       <c r="H58">
         <v>213</v>
       </c>
-      <c r="I58">
+      <c r="I58" s="3">
         <v>93.452197971103601</v>
       </c>
       <c r="J58">
@@ -3697,18 +3909,21 @@
         <v>0.34200000000000003</v>
       </c>
       <c r="P58" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B59" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C59" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D59">
         <v>206</v>
@@ -3716,7 +3931,7 @@
       <c r="E59">
         <v>20</v>
       </c>
-      <c r="F59">
+      <c r="F59" s="5">
         <v>91.150442477876098</v>
       </c>
       <c r="G59">
@@ -3725,7 +3940,7 @@
       <c r="H59">
         <v>213</v>
       </c>
-      <c r="I59">
+      <c r="I59" s="3">
         <v>93.452197971103601</v>
       </c>
       <c r="J59">
@@ -3747,18 +3962,21 @@
         <v>0.34200000000000003</v>
       </c>
       <c r="P59" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>98</v>
+      </c>
+      <c r="B60" t="s">
         <v>96</v>
       </c>
-      <c r="B60" t="s">
-        <v>94</v>
-      </c>
       <c r="C60" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D60">
         <v>197</v>
@@ -3766,7 +3984,7 @@
       <c r="E60">
         <v>12</v>
       </c>
-      <c r="F60">
+      <c r="F60" s="5">
         <v>94.258373205741634</v>
       </c>
       <c r="G60">
@@ -3775,7 +3993,7 @@
       <c r="H60">
         <v>213</v>
       </c>
-      <c r="I60">
+      <c r="I60" s="3">
         <v>93.452197971103601</v>
       </c>
       <c r="J60">
@@ -3797,18 +4015,21 @@
         <v>0.77200000000000002</v>
       </c>
       <c r="P60" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B61" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C61" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D61">
         <v>125</v>
@@ -3816,7 +4037,7 @@
       <c r="E61">
         <v>15</v>
       </c>
-      <c r="F61">
+      <c r="F61" s="5">
         <v>89.285714285714292</v>
       </c>
       <c r="G61">
@@ -3825,7 +4046,7 @@
       <c r="H61">
         <v>213</v>
       </c>
-      <c r="I61">
+      <c r="I61" s="3">
         <v>93.452197971103601</v>
       </c>
       <c r="J61">
@@ -3847,18 +4068,21 @@
         <v>0.34200000000000003</v>
       </c>
       <c r="P61" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>100</v>
+      </c>
+      <c r="B62" t="s">
+        <v>101</v>
+      </c>
+      <c r="C62" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>98</v>
-      </c>
-      <c r="B62" t="s">
-        <v>99</v>
-      </c>
-      <c r="C62" t="s">
-        <v>18</v>
       </c>
       <c r="D62">
         <v>9</v>
@@ -3866,7 +4090,7 @@
       <c r="E62">
         <v>1</v>
       </c>
-      <c r="F62">
+      <c r="F62" s="5">
         <v>90</v>
       </c>
       <c r="G62">
@@ -3875,7 +4099,7 @@
       <c r="H62">
         <v>46</v>
       </c>
-      <c r="I62">
+      <c r="I62" s="3">
         <v>88.58560794044665</v>
       </c>
       <c r="J62">
@@ -3897,18 +4121,21 @@
         <v>1</v>
       </c>
       <c r="P62" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q62" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B63" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C63" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D63">
         <v>18</v>
@@ -3916,7 +4143,7 @@
       <c r="E63">
         <v>2</v>
       </c>
-      <c r="F63">
+      <c r="F63" s="5">
         <v>90</v>
       </c>
       <c r="G63">
@@ -3925,7 +4152,7 @@
       <c r="H63">
         <v>46</v>
       </c>
-      <c r="I63">
+      <c r="I63" s="3">
         <v>88.58560794044665</v>
       </c>
       <c r="J63">
@@ -3947,18 +4174,21 @@
         <v>1</v>
       </c>
       <c r="P63" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>103</v>
+      </c>
+      <c r="B64" t="s">
         <v>101</v>
       </c>
-      <c r="B64" t="s">
-        <v>99</v>
-      </c>
       <c r="C64" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D64">
         <v>26</v>
@@ -3966,7 +4196,7 @@
       <c r="E64">
         <v>7</v>
       </c>
-      <c r="F64">
+      <c r="F64" s="5">
         <v>78.787878787878782</v>
       </c>
       <c r="G64">
@@ -3975,7 +4205,7 @@
       <c r="H64">
         <v>46</v>
       </c>
-      <c r="I64">
+      <c r="I64" s="3">
         <v>88.58560794044665</v>
       </c>
       <c r="J64">
@@ -3997,18 +4227,21 @@
         <v>0.33700000000000002</v>
       </c>
       <c r="P64" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q64" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B65" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C65" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D65">
         <v>4</v>
@@ -4016,7 +4249,7 @@
       <c r="E65">
         <v>3</v>
       </c>
-      <c r="F65">
+      <c r="F65" s="5">
         <v>57.142857142857139</v>
       </c>
       <c r="G65">
@@ -4025,7 +4258,7 @@
       <c r="H65">
         <v>46</v>
       </c>
-      <c r="I65">
+      <c r="I65" s="3">
         <v>88.58560794044665</v>
       </c>
       <c r="J65">
@@ -4047,18 +4280,21 @@
         <v>0.33700000000000002</v>
       </c>
       <c r="P65" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>105</v>
+      </c>
+      <c r="B66" t="s">
+        <v>106</v>
+      </c>
+      <c r="C66" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>103</v>
-      </c>
-      <c r="B66" t="s">
-        <v>104</v>
-      </c>
-      <c r="C66" t="s">
-        <v>18</v>
       </c>
       <c r="D66">
         <v>8</v>
@@ -4066,7 +4302,7 @@
       <c r="E66">
         <v>1</v>
       </c>
-      <c r="F66">
+      <c r="F66" s="5">
         <v>88.888888888888886</v>
       </c>
       <c r="G66">
@@ -4075,7 +4311,7 @@
       <c r="H66">
         <v>69</v>
       </c>
-      <c r="I66">
+      <c r="I66" s="3">
         <v>76.923076923076934</v>
       </c>
       <c r="J66">
@@ -4097,18 +4333,21 @@
         <v>0.86199999999999999</v>
       </c>
       <c r="P66" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q66" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B67" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C67" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D67">
         <v>13</v>
@@ -4116,7 +4355,7 @@
       <c r="E67">
         <v>4</v>
       </c>
-      <c r="F67">
+      <c r="F67" s="5">
         <v>76.470588235294116</v>
       </c>
       <c r="G67">
@@ -4125,7 +4364,7 @@
       <c r="H67">
         <v>69</v>
       </c>
-      <c r="I67">
+      <c r="I67" s="3">
         <v>76.923076923076934</v>
       </c>
       <c r="J67">
@@ -4147,18 +4386,21 @@
         <v>1</v>
       </c>
       <c r="P67" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q67" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>108</v>
+      </c>
+      <c r="B68" t="s">
         <v>106</v>
       </c>
-      <c r="B68" t="s">
-        <v>104</v>
-      </c>
       <c r="C68" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D68">
         <v>25</v>
@@ -4166,7 +4408,7 @@
       <c r="E68">
         <v>4</v>
       </c>
-      <c r="F68">
+      <c r="F68" s="5">
         <v>86.206896551724128</v>
       </c>
       <c r="G68">
@@ -4175,7 +4417,7 @@
       <c r="H68">
         <v>69</v>
       </c>
-      <c r="I68">
+      <c r="I68" s="3">
         <v>76.923076923076934</v>
       </c>
       <c r="J68">
@@ -4197,18 +4439,21 @@
         <v>0.86199999999999999</v>
       </c>
       <c r="P68" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B69" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C69" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D69">
         <v>6</v>
@@ -4216,7 +4461,7 @@
       <c r="E69">
         <v>3</v>
       </c>
-      <c r="F69">
+      <c r="F69" s="5">
         <v>66.666666666666657</v>
       </c>
       <c r="G69">
@@ -4225,7 +4470,7 @@
       <c r="H69">
         <v>69</v>
       </c>
-      <c r="I69">
+      <c r="I69" s="3">
         <v>76.923076923076934</v>
       </c>
       <c r="J69">
@@ -4247,18 +4492,21 @@
         <v>0.86199999999999999</v>
       </c>
       <c r="P69" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q69" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>110</v>
+      </c>
+      <c r="B70" t="s">
+        <v>111</v>
+      </c>
+      <c r="C70" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>108</v>
-      </c>
-      <c r="B70" t="s">
-        <v>109</v>
-      </c>
-      <c r="C70" t="s">
-        <v>18</v>
       </c>
       <c r="D70">
         <v>26</v>
@@ -4266,7 +4514,7 @@
       <c r="E70">
         <v>4</v>
       </c>
-      <c r="F70">
+      <c r="F70" s="5">
         <v>86.666666666666671</v>
       </c>
       <c r="G70">
@@ -4275,7 +4523,7 @@
       <c r="H70">
         <v>187</v>
       </c>
-      <c r="I70">
+      <c r="I70" s="3">
         <v>88.666666666666671</v>
       </c>
       <c r="J70">
@@ -4297,18 +4545,21 @@
         <v>0.96099999999999997</v>
       </c>
       <c r="P70" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q70" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B71" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C71" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D71">
         <v>95</v>
@@ -4316,7 +4567,7 @@
       <c r="E71">
         <v>22</v>
       </c>
-      <c r="F71">
+      <c r="F71" s="5">
         <v>81.196581196581192</v>
       </c>
       <c r="G71">
@@ -4325,7 +4576,7 @@
       <c r="H71">
         <v>187</v>
       </c>
-      <c r="I71">
+      <c r="I71" s="3">
         <v>88.666666666666671</v>
       </c>
       <c r="J71">
@@ -4347,18 +4598,21 @@
         <v>0.249</v>
       </c>
       <c r="P71" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q71" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>113</v>
+      </c>
+      <c r="B72" t="s">
         <v>111</v>
       </c>
-      <c r="B72" t="s">
-        <v>109</v>
-      </c>
       <c r="C72" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D72">
         <v>99</v>
@@ -4366,7 +4620,7 @@
       <c r="E72">
         <v>17</v>
       </c>
-      <c r="F72">
+      <c r="F72" s="5">
         <v>85.34482758620689</v>
       </c>
       <c r="G72">
@@ -4375,7 +4629,7 @@
       <c r="H72">
         <v>187</v>
       </c>
-      <c r="I72">
+      <c r="I72" s="3">
         <v>88.666666666666671</v>
       </c>
       <c r="J72">
@@ -4397,18 +4651,21 @@
         <v>0.96099999999999997</v>
       </c>
       <c r="P72" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q72" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B73" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C73" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D73">
         <v>72</v>
@@ -4416,7 +4673,7 @@
       <c r="E73">
         <v>10</v>
       </c>
-      <c r="F73">
+      <c r="F73" s="5">
         <v>87.804878048780495</v>
       </c>
       <c r="G73">
@@ -4425,7 +4682,7 @@
       <c r="H73">
         <v>187</v>
       </c>
-      <c r="I73">
+      <c r="I73" s="3">
         <v>88.666666666666671</v>
       </c>
       <c r="J73">
@@ -4447,18 +4704,21 @@
         <v>0.96099999999999997</v>
       </c>
       <c r="P73" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>115</v>
+      </c>
+      <c r="B74" t="s">
+        <v>116</v>
+      </c>
+      <c r="C74" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>113</v>
-      </c>
-      <c r="B74" t="s">
-        <v>114</v>
-      </c>
-      <c r="C74" t="s">
-        <v>18</v>
       </c>
       <c r="D74">
         <v>3</v>
@@ -4466,7 +4726,7 @@
       <c r="E74">
         <v>0</v>
       </c>
-      <c r="F74">
+      <c r="F74" s="5">
         <v>100</v>
       </c>
       <c r="G74">
@@ -4475,14 +4735,14 @@
       <c r="H74">
         <v>9</v>
       </c>
-      <c r="I74">
+      <c r="I74" s="3">
         <v>93.382352941176478</v>
       </c>
       <c r="J74">
         <v>139</v>
       </c>
       <c r="K74" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L74">
         <v>1</v>
@@ -4491,24 +4751,27 @@
         <v>2.6567478535029169E-2</v>
       </c>
       <c r="N74" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O74">
         <v>1</v>
       </c>
       <c r="P74" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q74" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B75" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C75" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D75">
         <v>6</v>
@@ -4516,7 +4779,7 @@
       <c r="E75">
         <v>0</v>
       </c>
-      <c r="F75">
+      <c r="F75" s="5">
         <v>100</v>
       </c>
       <c r="G75">
@@ -4525,14 +4788,14 @@
       <c r="H75">
         <v>9</v>
       </c>
-      <c r="I75">
+      <c r="I75" s="3">
         <v>93.382352941176478</v>
       </c>
       <c r="J75">
         <v>142</v>
       </c>
       <c r="K75" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L75">
         <v>1</v>
@@ -4541,24 +4804,27 @@
         <v>7.1609713208776002E-2</v>
       </c>
       <c r="N75" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O75">
         <v>1</v>
       </c>
       <c r="P75" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q75" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>118</v>
+      </c>
+      <c r="B76" t="s">
         <v>116</v>
       </c>
-      <c r="B76" t="s">
-        <v>114</v>
-      </c>
       <c r="C76" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D76">
         <v>10</v>
@@ -4566,7 +4832,7 @@
       <c r="E76">
         <v>0</v>
       </c>
-      <c r="F76">
+      <c r="F76" s="5">
         <v>100</v>
       </c>
       <c r="G76">
@@ -4575,14 +4841,14 @@
       <c r="H76">
         <v>9</v>
       </c>
-      <c r="I76">
+      <c r="I76" s="3">
         <v>93.382352941176478</v>
       </c>
       <c r="J76">
         <v>146</v>
       </c>
       <c r="K76" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L76">
         <v>1</v>
@@ -4591,24 +4857,27 @@
         <v>0.13244640464149959</v>
       </c>
       <c r="N76" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O76">
         <v>1</v>
       </c>
       <c r="P76" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q76" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B77" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C77" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D77">
         <v>34</v>
@@ -4616,7 +4885,7 @@
       <c r="E77">
         <v>5</v>
       </c>
-      <c r="F77">
+      <c r="F77" s="5">
         <v>87.179487179487182</v>
       </c>
       <c r="G77">
@@ -4625,7 +4894,7 @@
       <c r="H77">
         <v>9</v>
       </c>
-      <c r="I77">
+      <c r="I77" s="3">
         <v>93.382352941176478</v>
       </c>
       <c r="J77">
@@ -4647,18 +4916,21 @@
         <v>1</v>
       </c>
       <c r="P77" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q77" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>120</v>
+      </c>
+      <c r="B78" t="s">
+        <v>121</v>
+      </c>
+      <c r="C78" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>118</v>
-      </c>
-      <c r="B78" t="s">
-        <v>119</v>
-      </c>
-      <c r="C78" t="s">
-        <v>18</v>
       </c>
       <c r="D78">
         <v>18</v>
@@ -4666,7 +4938,7 @@
       <c r="E78">
         <v>2</v>
       </c>
-      <c r="F78">
+      <c r="F78" s="5">
         <v>90</v>
       </c>
       <c r="G78">
@@ -4675,7 +4947,7 @@
       <c r="H78">
         <v>162</v>
       </c>
-      <c r="I78">
+      <c r="I78" s="3">
         <v>85.232452142206014</v>
       </c>
       <c r="J78">
@@ -4697,18 +4969,21 @@
         <v>1</v>
       </c>
       <c r="P78" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q78" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B79" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C79" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D79">
         <v>26</v>
@@ -4716,7 +4991,7 @@
       <c r="E79">
         <v>3</v>
       </c>
-      <c r="F79">
+      <c r="F79" s="5">
         <v>89.65517241379311</v>
       </c>
       <c r="G79">
@@ -4725,7 +5000,7 @@
       <c r="H79">
         <v>162</v>
       </c>
-      <c r="I79">
+      <c r="I79" s="3">
         <v>85.232452142206014</v>
       </c>
       <c r="J79">
@@ -4747,18 +5022,21 @@
         <v>1</v>
       </c>
       <c r="P79" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q79" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>123</v>
+      </c>
+      <c r="B80" t="s">
         <v>121</v>
       </c>
-      <c r="B80" t="s">
-        <v>119</v>
-      </c>
       <c r="C80" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D80">
         <v>88</v>
@@ -4766,7 +5044,7 @@
       <c r="E80">
         <v>24</v>
       </c>
-      <c r="F80">
+      <c r="F80" s="5">
         <v>78.571428571428569</v>
       </c>
       <c r="G80">
@@ -4775,7 +5053,7 @@
       <c r="H80">
         <v>162</v>
       </c>
-      <c r="I80">
+      <c r="I80" s="3">
         <v>85.232452142206014</v>
       </c>
       <c r="J80">
@@ -4797,18 +5075,21 @@
         <v>0.73099999999999998</v>
       </c>
       <c r="P80" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q80" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B81" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C81" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D81">
         <v>36</v>
@@ -4816,7 +5097,7 @@
       <c r="E81">
         <v>4</v>
       </c>
-      <c r="F81">
+      <c r="F81" s="5">
         <v>90</v>
       </c>
       <c r="G81">
@@ -4825,7 +5106,7 @@
       <c r="H81">
         <v>162</v>
       </c>
-      <c r="I81">
+      <c r="I81" s="3">
         <v>85.232452142206014</v>
       </c>
       <c r="J81">
@@ -4847,18 +5128,21 @@
         <v>1</v>
       </c>
       <c r="P81" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q81" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>125</v>
+      </c>
+      <c r="B82" t="s">
+        <v>126</v>
+      </c>
+      <c r="C82" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>123</v>
-      </c>
-      <c r="B82" t="s">
-        <v>124</v>
-      </c>
-      <c r="C82" t="s">
-        <v>18</v>
       </c>
       <c r="D82">
         <v>5</v>
@@ -4866,7 +5150,7 @@
       <c r="E82">
         <v>2</v>
       </c>
-      <c r="F82">
+      <c r="F82" s="5">
         <v>71.428571428571431</v>
       </c>
       <c r="G82">
@@ -4875,7 +5159,7 @@
       <c r="H82">
         <v>49</v>
       </c>
-      <c r="I82">
+      <c r="I82" s="3">
         <v>79.237288135593218</v>
       </c>
       <c r="J82">
@@ -4897,18 +5181,21 @@
         <v>1</v>
       </c>
       <c r="P82" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q82" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B83" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C83" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D83">
         <v>5</v>
@@ -4916,7 +5203,7 @@
       <c r="E83">
         <v>2</v>
       </c>
-      <c r="F83">
+      <c r="F83" s="5">
         <v>71.428571428571431</v>
       </c>
       <c r="G83">
@@ -4925,7 +5212,7 @@
       <c r="H83">
         <v>49</v>
       </c>
-      <c r="I83">
+      <c r="I83" s="3">
         <v>79.237288135593218</v>
       </c>
       <c r="J83">
@@ -4947,18 +5234,21 @@
         <v>1</v>
       </c>
       <c r="P83" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q83" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>128</v>
+      </c>
+      <c r="B84" t="s">
         <v>126</v>
       </c>
-      <c r="B84" t="s">
-        <v>124</v>
-      </c>
       <c r="C84" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D84">
         <v>13</v>
@@ -4966,7 +5256,7 @@
       <c r="E84">
         <v>7</v>
       </c>
-      <c r="F84">
+      <c r="F84" s="5">
         <v>65</v>
       </c>
       <c r="G84">
@@ -4975,7 +5265,7 @@
       <c r="H84">
         <v>49</v>
       </c>
-      <c r="I84">
+      <c r="I84" s="3">
         <v>79.237288135593218</v>
       </c>
       <c r="J84">
@@ -4997,18 +5287,21 @@
         <v>1</v>
       </c>
       <c r="P84" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q84" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B85" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C85" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D85">
         <v>8</v>
@@ -5016,7 +5309,7 @@
       <c r="E85">
         <v>3</v>
       </c>
-      <c r="F85">
+      <c r="F85" s="5">
         <v>72.727272727272734</v>
       </c>
       <c r="G85">
@@ -5025,7 +5318,7 @@
       <c r="H85">
         <v>49</v>
       </c>
-      <c r="I85">
+      <c r="I85" s="3">
         <v>79.237288135593218</v>
       </c>
       <c r="J85">
@@ -5047,18 +5340,21 @@
         <v>1</v>
       </c>
       <c r="P85" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q85" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>130</v>
+      </c>
+      <c r="B86" t="s">
+        <v>131</v>
+      </c>
+      <c r="C86" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>128</v>
-      </c>
-      <c r="B86" t="s">
-        <v>129</v>
-      </c>
-      <c r="C86" t="s">
-        <v>18</v>
       </c>
       <c r="D86">
         <v>28</v>
@@ -5066,7 +5362,7 @@
       <c r="E86">
         <v>4</v>
       </c>
-      <c r="F86">
+      <c r="F86" s="5">
         <v>87.5</v>
       </c>
       <c r="G86">
@@ -5075,7 +5371,7 @@
       <c r="H86">
         <v>243</v>
       </c>
-      <c r="I86">
+      <c r="I86" s="3">
         <v>85.370258880192651</v>
       </c>
       <c r="J86">
@@ -5097,18 +5393,21 @@
         <v>1</v>
       </c>
       <c r="P86" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q86" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B87" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C87" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D87">
         <v>85</v>
@@ -5116,7 +5415,7 @@
       <c r="E87">
         <v>12</v>
       </c>
-      <c r="F87">
+      <c r="F87" s="5">
         <v>87.628865979381445</v>
       </c>
       <c r="G87">
@@ -5125,7 +5424,7 @@
       <c r="H87">
         <v>243</v>
       </c>
-      <c r="I87">
+      <c r="I87" s="3">
         <v>85.370258880192651</v>
       </c>
       <c r="J87">
@@ -5147,18 +5446,21 @@
         <v>1</v>
       </c>
       <c r="P87" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q87" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>133</v>
+      </c>
+      <c r="B88" t="s">
         <v>131</v>
       </c>
-      <c r="B88" t="s">
-        <v>129</v>
-      </c>
       <c r="C88" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D88">
         <v>156</v>
@@ -5166,7 +5468,7 @@
       <c r="E88">
         <v>36</v>
       </c>
-      <c r="F88">
+      <c r="F88" s="5">
         <v>81.25</v>
       </c>
       <c r="G88">
@@ -5175,7 +5477,7 @@
       <c r="H88">
         <v>243</v>
       </c>
-      <c r="I88">
+      <c r="I88" s="3">
         <v>85.370258880192651</v>
       </c>
       <c r="J88">
@@ -5197,18 +5499,21 @@
         <v>0.92500000000000004</v>
       </c>
       <c r="P88" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q88" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B89" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C89" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D89">
         <v>33</v>
@@ -5216,7 +5521,7 @@
       <c r="E89">
         <v>7</v>
       </c>
-      <c r="F89">
+      <c r="F89" s="5">
         <v>82.5</v>
       </c>
       <c r="G89">
@@ -5225,7 +5530,7 @@
       <c r="H89">
         <v>243</v>
       </c>
-      <c r="I89">
+      <c r="I89" s="3">
         <v>85.370258880192651</v>
       </c>
       <c r="J89">
@@ -5247,18 +5552,21 @@
         <v>1</v>
       </c>
       <c r="P89" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q89" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>135</v>
+      </c>
+      <c r="B90" t="s">
+        <v>136</v>
+      </c>
+      <c r="C90" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>133</v>
-      </c>
-      <c r="B90" t="s">
-        <v>134</v>
-      </c>
-      <c r="C90" t="s">
-        <v>18</v>
       </c>
       <c r="D90">
         <v>15</v>
@@ -5266,7 +5574,7 @@
       <c r="E90">
         <v>1</v>
       </c>
-      <c r="F90">
+      <c r="F90" s="5">
         <v>93.75</v>
       </c>
       <c r="G90">
@@ -5275,7 +5583,7 @@
       <c r="H90">
         <v>58</v>
       </c>
-      <c r="I90">
+      <c r="I90" s="3">
         <v>88.353413654618478</v>
       </c>
       <c r="J90">
@@ -5297,18 +5605,21 @@
         <v>1</v>
       </c>
       <c r="P90" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q90" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B91" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C91" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D91">
         <v>16</v>
@@ -5316,7 +5627,7 @@
       <c r="E91">
         <v>1</v>
       </c>
-      <c r="F91">
+      <c r="F91" s="5">
         <v>94.117647058823522</v>
       </c>
       <c r="G91">
@@ -5325,7 +5636,7 @@
       <c r="H91">
         <v>58</v>
       </c>
-      <c r="I91">
+      <c r="I91" s="3">
         <v>88.353413654618478</v>
       </c>
       <c r="J91">
@@ -5347,18 +5658,21 @@
         <v>1</v>
       </c>
       <c r="P91" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q91" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>138</v>
+      </c>
+      <c r="B92" t="s">
         <v>136</v>
       </c>
-      <c r="B92" t="s">
-        <v>134</v>
-      </c>
       <c r="C92" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D92">
         <v>47</v>
@@ -5366,7 +5680,7 @@
       <c r="E92">
         <v>7</v>
       </c>
-      <c r="F92">
+      <c r="F92" s="5">
         <v>87.037037037037038</v>
       </c>
       <c r="G92">
@@ -5375,7 +5689,7 @@
       <c r="H92">
         <v>58</v>
       </c>
-      <c r="I92">
+      <c r="I92" s="3">
         <v>88.353413654618478</v>
       </c>
       <c r="J92">
@@ -5397,18 +5711,21 @@
         <v>1</v>
       </c>
       <c r="P92" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="Q92" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B93" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C93" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D93">
         <v>11</v>
@@ -5416,7 +5733,7 @@
       <c r="E93">
         <v>0</v>
       </c>
-      <c r="F93">
+      <c r="F93" s="5">
         <v>100</v>
       </c>
       <c r="G93">
@@ -5425,14 +5742,14 @@
       <c r="H93">
         <v>58</v>
       </c>
-      <c r="I93">
+      <c r="I93" s="3">
         <v>88.353413654618478</v>
       </c>
       <c r="J93">
         <v>509</v>
       </c>
       <c r="K93" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L93">
         <v>0.623</v>
@@ -5441,13 +5758,16 @@
         <v>0.3210136993721327</v>
       </c>
       <c r="N93" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O93">
         <v>1</v>
       </c>
       <c r="P93" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="Q93" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>